<commit_message>
Excel for Mac's answers to looks-ru (ru-RU: 79 of 80 looks as predicted, the miss Excel for Mac's order of Latin after Cyrillic) and files again, without the average rule with equal and deviations, which is no input now; rules compared by meaning (cells as a set, canonical formulas, a format as its code)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/cond/files/kinds-delete-col.xlsx
+++ b/test/excel/cond/files/kinds-delete-col.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fcond-43137/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fcond-66268/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BD3BE8D-7288-9E4F-8D16-105062197BC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{865F52FA-FEA2-0B42-B1E4-AC45E981FC3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1070,7 +1070,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:D11">
     <cfRule type="top10" dxfId="5" priority="9" percent="1" bottom="1" rank="30"/>
-    <cfRule type="aboveAverage" dxfId="4" priority="10" aboveAverage="0" equalAverage="1"/>
+    <cfRule type="aboveAverage" dxfId="4" priority="10" aboveAverage="0" stdDev="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1:E11">
     <cfRule type="uniqueValues" dxfId="3" priority="11"/>

</xml_diff>